<commit_message>
LORANI B5 : métré contre DPGF dans le contrôle du dossier (b5_16 amendé avant pose : rôle metre, nature metre_dpgf, écart > 5 %, sous-estimé > 10 % majeur) ; type lorani_metre ; test b5_07 § 10 ; écran, rapport, exemple
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018iNiXjY8eWmMjaGrXSGgma
</commit_message>
<xml_diff>
--- a/omega/recette-b5/rapport-controle-exemple.xlsx
+++ b/omega/recette-b5/rapport-controle-exemple.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Pièces" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Constats!$A$1:$N$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Constats!$A$1:$N$10</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -268,42 +268,40 @@
       </c>
       <c r="B4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Mineur</t>
+          <t xml:space="preserve">Majeur</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CCTP et DPGF</t>
+          <t xml:space="preserve">Métré et DPGF</t>
         </is>
       </c>
       <c r="D4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Le poste 2.4 « Isolation thermique par l'extérieur » est décrit au CCTP (CCTP 02, p. 9) mais n'est pas chiffré à la DPGF.</t>
+          <t xml:space="preserve">Le poste 2.2 est chiffré à 64 m2 à la DPGF (DPGF 02, p. 1) pour 78,4 m2 mesurés (PC2, p. 1 ; PC3, p. 1) : sous-estimé de 18 %.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ajouter le poste 2.4 à la DPGF, ou le retirer du CCTP.</t>
+          <t xml:space="preserve">Porter la quantité du poste 2.2 à 78,4 m2 à la DPGF, ou justifier l'écart.</t>
         </is>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CCTP 02</t>
+          <t xml:space="preserve">PC2</t>
         </is>
       </c>
       <c r="H4" s="2">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="I4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2.4 Isolation thermique par l'extérieur (ITE)</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Isolation thermique par l'extérieur</t>
-        </is>
+          <t xml:space="preserve">Dalle haute R+3 : 52,60 m²</t>
+        </is>
+      </c>
+      <c r="J4" s="2">
+        <v>52.6</v>
       </c>
       <c r="K4" t="inlineStr" s="2">
         <is>
@@ -320,162 +318,326 @@
     </row>
     <row r="5">
       <c r="A5" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Mineur</t>
+          <t xml:space="preserve">Majeur</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CCTP et DPGF</t>
+          <t xml:space="preserve">Métré et DPGF</t>
         </is>
       </c>
       <c r="D5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Le poste 2.7 est chiffré à la DPGF (DPGF 02, p. 2) sans description au CCTP.</t>
+          <t xml:space="preserve">Le poste 2.2 est chiffré à 64 m2 à la DPGF (DPGF 02, p. 1) pour 78,4 m2 mesurés (PC2, p. 1 ; PC3, p. 1) : sous-estimé de 18 %.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Décrire le poste 2.7 au CCTP, ou le retirer de la DPGF.</t>
+          <t xml:space="preserve">Porter la quantité du poste 2.2 à 78,4 m2 à la DPGF, ou justifier l'écart.</t>
         </is>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">PC3</t>
+        </is>
+      </c>
+      <c r="H5" s="2">
+        <v>1</v>
+      </c>
+      <c r="I5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Terrasse : 25,80 m²</t>
+        </is>
+      </c>
+      <c r="J5" s="2">
+        <v>25.8</v>
+      </c>
+      <c r="K5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Ouvert</t>
+        </is>
+      </c>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2">
+        <v>2</v>
+      </c>
+      <c r="B6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Majeur</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Métré et DPGF</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Le poste 2.2 est chiffré à 64 m2 à la DPGF (DPGF 02, p. 1) pour 78,4 m2 mesurés (PC2, p. 1 ; PC3, p. 1) : sous-estimé de 18 %.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Porter la quantité du poste 2.2 à 78,4 m2 à la DPGF, ou justifier l'écart.</t>
+        </is>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">DPGF 02</t>
         </is>
       </c>
-      <c r="H5" s="2">
-        <v>2</v>
-      </c>
-      <c r="I5" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">2.7 Garde-corps terrasse — option — ens 1</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Écarté</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Option chiffrée à part, à la demande du maître d'ouvrage.</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Vous</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">oui</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2"/>
-      <c r="B6" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Majeur</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Entre les planches</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">La hauteur au faîtage diffère d'une pièce à l'autre : 15,6 m sur PC3 (p. 1) ; 16,1 m sur PC5 (p. 1).</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Aligner la hauteur au faîtage sur une seule valeur dans toutes les pièces (écart de 0,5 m). Valeur la plus fréquente : 15,6 m.</t>
-        </is>
-      </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
+      <c r="H6" s="2">
+        <v>1</v>
+      </c>
+      <c r="I6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">2.2 Plancher béton R+3 — m2 — 64,00</t>
+        </is>
+      </c>
+      <c r="J6" s="2">
+        <v>64</v>
+      </c>
       <c r="K6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Corrigé à l'indice B</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Corrigé à l'indice B.</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Ouvert</t>
+        </is>
+      </c>
+      <c r="L6" s="2"/>
       <c r="M6" s="2"/>
       <c r="N6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">indice A</t>
+          <t xml:space="preserve">oui</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2"/>
+      <c r="A7" s="2">
+        <v>3</v>
+      </c>
       <c r="B7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Bloquant</t>
+          <t xml:space="preserve">Mineur</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Contre le PLU</t>
+          <t xml:space="preserve">CCTP et DPGF</t>
         </is>
       </c>
       <c r="D7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">La hauteur au faîtage (16,1 m sur PC5, p. 1) dépasse la règle du PLU (au plus 16 m, article URm1 10).</t>
+          <t xml:space="preserve">Le poste 2.4 « Isolation thermique par l'extérieur » est décrit au CCTP (CCTP 02, p. 9) mais n'est pas chiffré à la DPGF.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ramener la hauteur au faîtage à au plus 16 m (article URm1 10 du règlement), ou justifier une dérogation.</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">URm1 10</t>
-        </is>
-      </c>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
+          <t xml:space="preserve">Ajouter le poste 2.4 à la DPGF, ou le retirer du CCTP.</t>
+        </is>
+      </c>
+      <c r="F7" s="2"/>
+      <c r="G7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CCTP 02</t>
+        </is>
+      </c>
+      <c r="H7" s="2">
+        <v>9</v>
+      </c>
+      <c r="I7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">2.4 Isolation thermique par l'extérieur (ITE)</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Isolation thermique par l'extérieur</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Corrigé à l'indice B</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Corrigé à l'indice B.</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Ouvert</t>
+        </is>
+      </c>
+      <c r="L7" s="2"/>
       <c r="M7" s="2"/>
       <c r="N7" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2">
+        <v>4</v>
+      </c>
+      <c r="B8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Mineur</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CCTP et DPGF</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Le poste 2.7 est chiffré à la DPGF (DPGF 02, p. 2) sans description au CCTP.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Décrire le poste 2.7 au CCTP, ou le retirer de la DPGF.</t>
+        </is>
+      </c>
+      <c r="F8" s="2"/>
+      <c r="G8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">DPGF 02</t>
+        </is>
+      </c>
+      <c r="H8" s="2">
+        <v>2</v>
+      </c>
+      <c r="I8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">2.7 Garde-corps terrasse — option — ens 1</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Écarté</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Option chiffrée à part, à la demande du maître d'ouvrage.</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Vous</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2"/>
+      <c r="B9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Majeur</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Entre les planches</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">La hauteur au faîtage diffère d'une pièce à l'autre : 15,6 m sur PC3 (p. 1) ; 16,1 m sur PC5 (p. 1).</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aligner la hauteur au faîtage sur une seule valeur dans toutes les pièces (écart de 0,5 m). Valeur la plus fréquente : 15,6 m.</t>
+        </is>
+      </c>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Corrigé à l'indice B</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Corrigé à l'indice B.</t>
+        </is>
+      </c>
+      <c r="M9" s="2"/>
+      <c r="N9" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">indice A</t>
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2"/>
+      <c r="B10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Bloquant</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Contre le PLU</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">La hauteur au faîtage (16,1 m sur PC5, p. 1) dépasse la règle du PLU (au plus 16 m, article URm1 10).</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Ramener la hauteur au faîtage à au plus 16 m (article URm1 10 du règlement), ou justifier une dérogation.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">URm1 10</t>
+        </is>
+      </c>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Corrigé à l'indice B</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Corrigé à l'indice B.</t>
+        </is>
+      </c>
+      <c r="M10" s="2"/>
+      <c r="N10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">indice A</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N7"/>
+  <autoFilter ref="A1:N10"/>
 </worksheet>
 </file>
 

</xml_diff>